<commit_message>
fix(qc): improve sampling point mapping and diagnostics
</commit_message>
<xml_diff>
--- a/domains/qc/doc/Master-Data.xlsx
+++ b/domains/qc/doc/Master-Data.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameter" sheetId="1" r:id="R45335e2185354f7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sampling-Point" sheetId="2" r:id="R0aab524b38ea41eb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parameter" sheetId="1" r:id="R7583249bc54f483e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sampling-Point" sheetId="2" r:id="R66d48957ad074dc2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2770,7 +2770,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21be9adc95844fdb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ab7a0f15b6d4faa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2816,7 +2816,7 @@
         <x:v>Octanol</x:v>
       </x:c>
       <x:c r="F2" s="21" t="n">
-        <x:v>59</x:v>
+        <x:v>61</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -2938,7 +2938,7 @@
         <x:v>Total Sampling Point</x:v>
       </x:c>
       <x:c r="F9" s="21" t="n">
-        <x:v>191</x:v>
+        <x:v>193</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -5326,12 +5326,8 @@
       <x:c r="F186"/>
     </x:row>
     <x:row r="187">
-      <x:c r="A187" s="11" t="str">
-        <x:v>NPG</x:v>
-      </x:c>
-      <x:c r="B187" s="11" t="str">
-        <x:v>NPG FLAKER</x:v>
-      </x:c>
+      <x:c r="A187" s="11"/>
+      <x:c r="B187" s="11"/>
       <x:c r="C187" s="11"/>
       <x:c r="D187"/>
       <x:c r="E187"/>
@@ -5583,10 +5579,34 @@
       <x:c r="E206"/>
       <x:c r="F206"/>
     </x:row>
+    <x:row r="207">
+      <x:c r="A207" t="str">
+        <x:v>Octanol</x:v>
+      </x:c>
+      <x:c r="B207" t="str">
+        <x:v>T-170 MIDDLE</x:v>
+      </x:c>
+      <x:c r="C207"/>
+      <x:c r="D207"/>
+      <x:c r="E207"/>
+      <x:c r="F207"/>
+    </x:row>
+    <x:row r="208">
+      <x:c r="A208" t="str">
+        <x:v>Octanol</x:v>
+      </x:c>
+      <x:c r="B208" t="str">
+        <x:v>TK-172</x:v>
+      </x:c>
+      <x:c r="C208"/>
+      <x:c r="D208"/>
+      <x:c r="E208"/>
+      <x:c r="F208"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R17c073084611470b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Refa5aa8eaa4543d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>